<commit_message>
fix(quick-report): mirror 3-tier date folders in CLI and output
Selection was picking station level only, causing batch generation across all dates into root QUICK REPORT/ folder. Use select_pahang_date_folder for 3-tier selection and mirror QUICK REPORT/<STATION>/<MONTH>/<DATE>/ output path hierarchy.
</commit_message>
<xml_diff>
--- a/templates/TOTAL PE.xlsx
+++ b/templates/TOTAL PE.xlsx
@@ -3523,7 +3523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.28515625" bestFit="1" customWidth="1" style="20" min="2" max="2"/>
@@ -3569,17 +3569,6 @@
       <c r="I1">
         <f t="array" ref="I1">_xlfn.TEXTJOIN(",", TRUE, _xlfn._xlws.FILTER(B:B, D:D=G1))</f>
         <v/>
-      </c>
-    </row>
-    <row r="2">
-      <c r="D2" s="10" t="n"/>
-    </row>
-    <row r="3">
-      <c r="D3" s="10" t="n"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>PASTE HERE AS TEXT</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>